<commit_message>
Add realistic body text to sample_articles.xlsx
The text column was empty; every row now has a 2-3 sentence article
body. Re-verified all 24 expected_is_epu labels against the real
production dictionary (unchanged) and re-executed test_with_excel.ipynb
end to end with zero errors.
</commit_message>
<xml_diff>
--- a/examples/sample_articles.xlsx
+++ b/examples/sample_articles.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="113">
   <si>
     <t>country</t>
   </si>
@@ -218,6 +218,78 @@
   </si>
   <si>
     <t>https://example.com/kenya/the-star/2024-02/03</t>
+  </si>
+  <si>
+    <t>The naira weakened further against the dollar on Monday as traders pointed to persistent inflation and a lack of clarity over the government's next fiscal policy move. Analysts said the uncertainty was keeping foreign investors on the sidelines.</t>
+  </si>
+  <si>
+    <t>The government on Monday unveiled a new tax reform package it says will boost economic growth over the next three years. Officials said the measures target small businesses and are expected to take effect from next quarter.</t>
+  </si>
+  <si>
+    <t>Thousands of fans packed the stadium on Sunday as the home team lifted the trophy after a hard-fought final. The coach praised the squad's discipline throughout the season.</t>
+  </si>
+  <si>
+    <t>The Central Bank of Nigeria raised its benchmark interest rate on Tuesday, citing a volatile exchange rate and the need to defend the currency. The decision was announced after a closed-door meeting of the monetary committee.</t>
+  </si>
+  <si>
+    <t>Inflation slowed slightly last month, but traders said unresolved questions about fiscal policy are keeping markets volatile. Several analysts cautioned against reading too much into one month of data.</t>
+  </si>
+  <si>
+    <t>The president signed the long-debated law on Wednesday after months of back and forth in the National Assembly. Opposition lawmakers said they would continue to press for amendments in the coming session.</t>
+  </si>
+  <si>
+    <t>The fiscal deficit widened for a second straight quarter as the government grappled with a deepening policy crisis. Officials acknowledged the shortfall but declined to say how it would be closed.</t>
+  </si>
+  <si>
+    <t>The Ministry of Finance unveiled a new regulation on Thursday covering how banks report quarterly figures. Industry groups said they were reviewing the details before commenting further.</t>
+  </si>
+  <si>
+    <t>Traders flagged rising market risk on Friday, describing the investment climate as unstable after a volatile week of trading. Several funds said they were holding more cash than usual.</t>
+  </si>
+  <si>
+    <t>GDP growth slowed in the first quarter as the central bank's tighter monetary policy fed through to the wider economy. Economists linked the slowdown to broader instability in the region.</t>
+  </si>
+  <si>
+    <t>A new government decree on public spending has raised uncertainty over the size of this year's fiscal deficit, according to budget officials who briefed reporters on Monday.</t>
+  </si>
+  <si>
+    <t>The economy grew at a steady pace last quarter, according to figures released on Tuesday. Officials described the performance as consistent with earlier forecasts.</t>
+  </si>
+  <si>
+    <t>The shilling weakened against major currencies on Monday as inflation data came in higher than expected and investors cited ongoing fiscal policy uncertainty ahead of the budget statement.</t>
+  </si>
+  <si>
+    <t>A government decree introduced new legislation on public spending on Wednesday, formalising limits that had circulated in draft form for weeks, officials said.</t>
+  </si>
+  <si>
+    <t>Athletes from across the region gathered on Saturday to prepare for next month's championship. Coaches said training camps would run through the rest of the month.</t>
+  </si>
+  <si>
+    <t>Foreign investment slowed in the first quarter as monetary policy tightened and the outlook for the rest of the year remained unclear, fund managers said on Thursday.</t>
+  </si>
+  <si>
+    <t>Economic growth slowed last quarter as new regulation and broader market uncertainty weighed on business confidence, a central bank survey found.</t>
+  </si>
+  <si>
+    <t>The Ministry of Finance said on Friday it was reviewing an earlier tax reform plan after feedback from industry groups during a public comment period.</t>
+  </si>
+  <si>
+    <t>GDP contracted in the latest quarter as the fiscal deficit widened further, with officials describing the outlook as unstable heading into the next budget cycle.</t>
+  </si>
+  <si>
+    <t>A new regulation on the exchange rate was introduced on Tuesday after weeks of unpredictable trading, the central bank said in a statement.</t>
+  </si>
+  <si>
+    <t>A new stadium opened downtown on Saturday with a friendly match between two local clubs. City officials said the venue would also host concerts later in the year.</t>
+  </si>
+  <si>
+    <t>Rising inflation and unresolved fiscal policy questions have created uncertainty for investors, several brokerages said in notes to clients on Wednesday.</t>
+  </si>
+  <si>
+    <t>New legislation on public spending and the fiscal deficit has left the budget outlook unclear, according to two lawmakers who spoke to reporters after Thursday's session.</t>
+  </si>
+  <si>
+    <t>The economy showed further signs of recovery last month, with retail sales and manufacturing output both picking up, a trade body said on Friday.</t>
   </si>
   <si>
     <t>naira(E) inflation(E) fiscal policy(P) uncertainty(U)</t>
@@ -696,11 +768,14 @@
       <c r="E2" s="2" t="s">
         <v>44</v>
       </c>
+      <c r="F2" t="s">
+        <v>68</v>
+      </c>
       <c r="G2" t="b">
         <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>68</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -719,11 +794,14 @@
       <c r="E3" s="2" t="s">
         <v>45</v>
       </c>
+      <c r="F3" t="s">
+        <v>69</v>
+      </c>
       <c r="G3" t="b">
         <v>0</v>
       </c>
       <c r="H3" t="s">
-        <v>69</v>
+        <v>93</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -742,11 +820,14 @@
       <c r="E4" s="2" t="s">
         <v>46</v>
       </c>
+      <c r="F4" t="s">
+        <v>70</v>
+      </c>
       <c r="G4" t="b">
         <v>0</v>
       </c>
       <c r="H4" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -765,11 +846,14 @@
       <c r="E5" s="2" t="s">
         <v>47</v>
       </c>
+      <c r="F5" t="s">
+        <v>71</v>
+      </c>
       <c r="G5" t="b">
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>71</v>
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -788,11 +872,14 @@
       <c r="E6" s="2" t="s">
         <v>48</v>
       </c>
+      <c r="F6" t="s">
+        <v>72</v>
+      </c>
       <c r="G6" t="b">
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>72</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -811,11 +898,14 @@
       <c r="E7" s="2" t="s">
         <v>49</v>
       </c>
+      <c r="F7" t="s">
+        <v>73</v>
+      </c>
       <c r="G7" t="b">
         <v>0</v>
       </c>
       <c r="H7" t="s">
-        <v>73</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -834,11 +924,14 @@
       <c r="E8" s="2" t="s">
         <v>50</v>
       </c>
+      <c r="F8" t="s">
+        <v>74</v>
+      </c>
       <c r="G8" t="b">
         <v>1</v>
       </c>
       <c r="H8" t="s">
-        <v>74</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -857,11 +950,14 @@
       <c r="E9" s="2" t="s">
         <v>51</v>
       </c>
+      <c r="F9" t="s">
+        <v>75</v>
+      </c>
       <c r="G9" t="b">
         <v>0</v>
       </c>
       <c r="H9" t="s">
-        <v>75</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -880,11 +976,14 @@
       <c r="E10" s="2" t="s">
         <v>52</v>
       </c>
+      <c r="F10" t="s">
+        <v>76</v>
+      </c>
       <c r="G10" t="b">
         <v>0</v>
       </c>
       <c r="H10" t="s">
-        <v>76</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -903,11 +1002,14 @@
       <c r="E11" s="2" t="s">
         <v>53</v>
       </c>
+      <c r="F11" t="s">
+        <v>77</v>
+      </c>
       <c r="G11" t="b">
         <v>1</v>
       </c>
       <c r="H11" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -926,11 +1028,14 @@
       <c r="E12" s="2" t="s">
         <v>54</v>
       </c>
+      <c r="F12" t="s">
+        <v>78</v>
+      </c>
       <c r="G12" t="b">
         <v>1</v>
       </c>
       <c r="H12" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -949,11 +1054,14 @@
       <c r="E13" s="2" t="s">
         <v>55</v>
       </c>
+      <c r="F13" t="s">
+        <v>79</v>
+      </c>
       <c r="G13" t="b">
         <v>0</v>
       </c>
       <c r="H13" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
     </row>
     <row r="14" spans="1:8">
@@ -972,11 +1080,14 @@
       <c r="E14" s="2" t="s">
         <v>56</v>
       </c>
+      <c r="F14" t="s">
+        <v>80</v>
+      </c>
       <c r="G14" t="b">
         <v>1</v>
       </c>
       <c r="H14" t="s">
-        <v>80</v>
+        <v>104</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -995,11 +1106,14 @@
       <c r="E15" s="2" t="s">
         <v>57</v>
       </c>
+      <c r="F15" t="s">
+        <v>81</v>
+      </c>
       <c r="G15" t="b">
         <v>0</v>
       </c>
       <c r="H15" t="s">
-        <v>81</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1018,11 +1132,14 @@
       <c r="E16" s="2" t="s">
         <v>58</v>
       </c>
+      <c r="F16" t="s">
+        <v>82</v>
+      </c>
       <c r="G16" t="b">
         <v>0</v>
       </c>
       <c r="H16" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1041,11 +1158,14 @@
       <c r="E17" s="2" t="s">
         <v>59</v>
       </c>
+      <c r="F17" t="s">
+        <v>83</v>
+      </c>
       <c r="G17" t="b">
         <v>1</v>
       </c>
       <c r="H17" t="s">
-        <v>82</v>
+        <v>106</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1064,11 +1184,14 @@
       <c r="E18" s="2" t="s">
         <v>60</v>
       </c>
+      <c r="F18" t="s">
+        <v>84</v>
+      </c>
       <c r="G18" t="b">
         <v>1</v>
       </c>
       <c r="H18" t="s">
-        <v>83</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1087,11 +1210,14 @@
       <c r="E19" s="2" t="s">
         <v>61</v>
       </c>
+      <c r="F19" t="s">
+        <v>85</v>
+      </c>
       <c r="G19" t="b">
         <v>0</v>
       </c>
       <c r="H19" t="s">
-        <v>84</v>
+        <v>108</v>
       </c>
     </row>
     <row r="20" spans="1:8">
@@ -1110,11 +1236,14 @@
       <c r="E20" s="2" t="s">
         <v>62</v>
       </c>
+      <c r="F20" t="s">
+        <v>86</v>
+      </c>
       <c r="G20" t="b">
         <v>0</v>
       </c>
       <c r="H20" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1133,11 +1262,14 @@
       <c r="E21" s="2" t="s">
         <v>63</v>
       </c>
+      <c r="F21" t="s">
+        <v>87</v>
+      </c>
       <c r="G21" t="b">
         <v>1</v>
       </c>
       <c r="H21" t="s">
-        <v>86</v>
+        <v>110</v>
       </c>
     </row>
     <row r="22" spans="1:8">
@@ -1156,11 +1288,14 @@
       <c r="E22" s="2" t="s">
         <v>64</v>
       </c>
+      <c r="F22" t="s">
+        <v>88</v>
+      </c>
       <c r="G22" t="b">
         <v>0</v>
       </c>
       <c r="H22" t="s">
-        <v>70</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1179,11 +1314,14 @@
       <c r="E23" s="2" t="s">
         <v>65</v>
       </c>
+      <c r="F23" t="s">
+        <v>89</v>
+      </c>
       <c r="G23" t="b">
         <v>1</v>
       </c>
       <c r="H23" t="s">
-        <v>87</v>
+        <v>111</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1202,11 +1340,14 @@
       <c r="E24" s="2" t="s">
         <v>66</v>
       </c>
+      <c r="F24" t="s">
+        <v>90</v>
+      </c>
       <c r="G24" t="b">
         <v>1</v>
       </c>
       <c r="H24" t="s">
-        <v>88</v>
+        <v>112</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1225,11 +1366,14 @@
       <c r="E25" s="2" t="s">
         <v>67</v>
       </c>
+      <c r="F25" t="s">
+        <v>91</v>
+      </c>
       <c r="G25" t="b">
         <v>0</v>
       </c>
       <c r="H25" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>